<commit_message>
style: fix dark mode tabular view styling to match mockup
</commit_message>
<xml_diff>
--- a/database/2nd year/Core/2nd year Core week-1.xlsx
+++ b/database/2nd year/Core/2nd year Core week-1.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Naresh\Desktop\Class Scehdule Manager\class-schedule-app\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Naresh\Desktop\Class Scehdule Manager\class-schedule-app\database\2nd year\Core\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8988F2A9-83AF-48AF-AEFE-2F662408B95D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17C0E686-E0AD-4509-9ACC-F2637E586EB1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>

</xml_diff>